<commit_message>
Add Debt Service Coverage as 12th KPI (v5): EBIT over interest plus scheduled principal (CPLTD/12), with dashboard grading, red-flag and narrative support, SQL parity in analysis_queries.sql and db.py, refreshed sample packet, and first unit tests (test_analyze.py, 9 tests)
</commit_message>
<xml_diff>
--- a/docs/sample_packet.xlsx
+++ b/docs/sample_packet.xlsx
@@ -20,7 +20,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Dashboard'!$1:$2</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="3">'Dashboard'!$A$1:$E$19</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">'Dashboard'!$A$1:$E$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2284,7 +2284,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2605,8 +2605,32 @@
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="14" t="inlineStr">
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>Debt Service Coverage</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C15" s="13" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D15" s="13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E15" s="13" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="F15" s="12" t="inlineStr">
+        <is>
+          <t>higher</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="14" t="inlineStr">
         <is>
           <t>How the grading scale works
 - Target: the goal for each KPI (edit freely).
@@ -2616,15 +2640,15 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19"/>
     <row r="20"/>
     <row r="21"/>
+    <row r="22"/>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A17:F21"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A18:F22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2637,7 +2661,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3032,13 +3056,37 @@
         </is>
       </c>
     </row>
+    <row r="20" ht="26" customHeight="1">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>Debt Service Coverage</t>
+        </is>
+      </c>
+      <c r="B20" s="25">
+        <f>IF(('P&amp;L'!B16+'Balance Sheet'!B19/12)=0,"N/A",('P&amp;L'!B19+'P&amp;L'!B16)/('P&amp;L'!B16+'Balance Sheet'!B19/12))</f>
+        <v/>
+      </c>
+      <c r="C20" s="26">
+        <f>Adjustments!B15</f>
+        <v/>
+      </c>
+      <c r="D20" s="22">
+        <f>IF(B20&gt;=Adjustments!$B$15,"A",IF(B20&gt;=Adjustments!$B$15-Adjustments!$C$15,"B",IF(B20&gt;=Adjustments!$B$15-Adjustments!$D$15,"C",IF(B20&gt;=Adjustments!$B$15-Adjustments!$E$15,"D","F"))))</f>
+        <v/>
+      </c>
+      <c r="E20" s="19" t="inlineStr">
+        <is>
+          <t>Earnings cover interest + scheduled principal (higher is better)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A3:E3"/>
   </mergeCells>
-  <conditionalFormatting sqref="D9:D19">
+  <conditionalFormatting sqref="D9:D20">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"A"</formula>
     </cfRule>
@@ -3067,7 +3115,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E75"/>
+  <dimension ref="A1:E76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -4230,48 +4278,56 @@
     <row r="70" ht="30" customHeight="1">
       <c r="A70" s="35" t="inlineStr">
         <is>
-          <t>•  Collections running at 7 days sales outstanding (on target).</t>
+          <t>•  Debt service coverage is 9.56x -- earnings cover interest plus scheduled principal 9.6 times over.</t>
         </is>
       </c>
     </row>
     <row r="71" ht="30" customHeight="1">
       <c r="A71" s="35" t="inlineStr">
         <is>
-          <t>•  Cash conversion cycle is 9 days (7 to collect + 9 of inventory - 7 to pay suppliers).</t>
+          <t>•  Collections running at 7 days sales outstanding (on target).</t>
         </is>
       </c>
     </row>
     <row r="72" ht="30" customHeight="1">
       <c r="A72" s="35" t="inlineStr">
         <is>
+          <t>•  Cash conversion cycle is 9 days (7 to collect + 9 of inventory - 7 to pay suppliers).</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="30" customHeight="1">
+      <c r="A73" s="35" t="inlineStr">
+        <is>
           <t>•  Against 2026 Budget, net income of $123,800 beat by 9.6% (budgeted $112,996).</t>
         </is>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" s="31" t="inlineStr">
+    <row r="75">
+      <c r="A75" s="31" t="inlineStr">
         <is>
           <t>Red flags</t>
         </is>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" s="36" t="inlineStr">
+    <row r="76">
+      <c r="A76" s="36" t="inlineStr">
         <is>
           <t>•  No red flags -- all clear.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="12">
     <mergeCell ref="A69:E69"/>
     <mergeCell ref="A65:E65"/>
+    <mergeCell ref="A73:E73"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A72:E72"/>
+    <mergeCell ref="A76:E76"/>
     <mergeCell ref="A68:E68"/>
     <mergeCell ref="A71:E71"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A75:E75"/>
     <mergeCell ref="A66:E66"/>
     <mergeCell ref="A70:E70"/>
     <mergeCell ref="A67:E67"/>

</xml_diff>